<commit_message>
Reconcile analytics outputs with source data
</commit_message>
<xml_diff>
--- a/outputs/analysis/advanced_analytics.xlsx
+++ b/outputs/analysis/advanced_analytics.xlsx
@@ -977,7 +977,7 @@
         <v>53</v>
       </c>
       <c r="F5">
-        <v>0.8325045429045878</v>
+        <v>0.8325045429045879</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1057,7 +1057,7 @@
         <v>54</v>
       </c>
       <c r="F9">
-        <v>0.7906190758627345</v>
+        <v>0.7906190758627342</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1077,7 +1077,7 @@
         <v>54</v>
       </c>
       <c r="F10">
-        <v>0.7667258950033126</v>
+        <v>0.7667258950033127</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1237,7 +1237,7 @@
         <v>53</v>
       </c>
       <c r="F18">
-        <v>0.7009191532278335</v>
+        <v>0.7009191532278334</v>
       </c>
     </row>
     <row r="19" spans="1:6">

</xml_diff>

<commit_message>
Add validation and fully reconcile analytics artifacts
</commit_message>
<xml_diff>
--- a/outputs/analysis/advanced_analytics.xlsx
+++ b/outputs/analysis/advanced_analytics.xlsx
@@ -917,7 +917,7 @@
         <v>52</v>
       </c>
       <c r="F2">
-        <v>0.8393138291805023</v>
+        <v>0.8393138291805022</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -937,7 +937,7 @@
         <v>52</v>
       </c>
       <c r="F3">
-        <v>0.8393138291805023</v>
+        <v>0.8393138291805022</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -957,7 +957,7 @@
         <v>52</v>
       </c>
       <c r="F4">
-        <v>0.8393138291805023</v>
+        <v>0.8393138291805022</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -977,7 +977,7 @@
         <v>53</v>
       </c>
       <c r="F5">
-        <v>0.8325045429045879</v>
+        <v>0.8325045429045881</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1057,7 +1057,7 @@
         <v>54</v>
       </c>
       <c r="F9">
-        <v>0.7906190758627342</v>
+        <v>0.7906190758627344</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1077,7 +1077,7 @@
         <v>54</v>
       </c>
       <c r="F10">
-        <v>0.7667258950033127</v>
+        <v>0.7667258950033126</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1237,7 +1237,7 @@
         <v>53</v>
       </c>
       <c r="F18">
-        <v>0.7009191532278334</v>
+        <v>0.7009191532278335</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -1257,7 +1257,7 @@
         <v>53</v>
       </c>
       <c r="F19">
-        <v>0.6916482120854045</v>
+        <v>0.6916482120854046</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -1277,7 +1277,7 @@
         <v>53</v>
       </c>
       <c r="F20">
-        <v>0.6916482120854045</v>
+        <v>0.6916482120854046</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -1297,7 +1297,7 @@
         <v>53</v>
       </c>
       <c r="F21">
-        <v>0.6916482120854045</v>
+        <v>0.6916482120854046</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revamp dashboard and fix audit issues
</commit_message>
<xml_diff>
--- a/outputs/analysis/advanced_analytics.xlsx
+++ b/outputs/analysis/advanced_analytics.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="118">
   <si>
     <t>feature</t>
   </si>
@@ -41,9 +41,6 @@
     <t>segment__c</t>
   </si>
   <si>
-    <t>campaign_impressions</t>
-  </si>
-  <si>
     <t>numberofemployees</t>
   </si>
   <si>
@@ -53,15 +50,9 @@
     <t>annualrevenue</t>
   </si>
   <si>
-    <t>email_opens</t>
-  </si>
-  <si>
     <t>director_contacts</t>
   </si>
   <si>
-    <t>email_clicks</t>
-  </si>
-  <si>
     <t>vp_contacts</t>
   </si>
   <si>
@@ -77,12 +68,6 @@
     <t>account6qa6sense__c</t>
   </si>
   <si>
-    <t>web_goal_completions</t>
-  </si>
-  <si>
-    <t>campaign_form_fills</t>
-  </si>
-  <si>
     <t>_opportunity_id</t>
   </si>
   <si>
@@ -92,85 +77,91 @@
     <t>win_probability</t>
   </si>
   <si>
+    <t>006UW000007kI4MYAU</t>
+  </si>
+  <si>
     <t>006f200001z0iZPAAY</t>
   </si>
   <si>
+    <t>006f20000200EsTAAU</t>
+  </si>
+  <si>
     <t>006f200001ym6iOAAQ</t>
   </si>
   <si>
-    <t>006f20000200EsTAAU</t>
-  </si>
-  <si>
-    <t>006UW000007kI4MYAU</t>
+    <t>006UW00000I6EagYAF</t>
   </si>
   <si>
     <t>006UW00000HVmjJYAT</t>
   </si>
   <si>
+    <t>006f200001x6cLUAAY</t>
+  </si>
+  <si>
     <t>006f200001x7lFDAAY</t>
   </si>
   <si>
-    <t>006f200001x6cLUAAY</t>
-  </si>
-  <si>
-    <t>006UW00000I6EagYAF</t>
-  </si>
-  <si>
     <t>006f200001zznOJAAY</t>
   </si>
   <si>
+    <t>006UW00000J957BYAR</t>
+  </si>
+  <si>
+    <t>006UW00000J8n2MYAR</t>
+  </si>
+  <si>
+    <t>006UW00000J8xxeYAB</t>
+  </si>
+  <si>
+    <t>006UW00000J8vsdYAB</t>
+  </si>
+  <si>
+    <t>006UW00000J8onuYAB</t>
+  </si>
+  <si>
+    <t>006UW00000J8z3OYAR</t>
+  </si>
+  <si>
+    <t>006UW00000I6MczYAF</t>
+  </si>
+  <si>
+    <t>006f200001xUsIBAA0</t>
+  </si>
+  <si>
+    <t>006f200001yljUZAAY</t>
+  </si>
+  <si>
     <t>0064P00000ySq9bQAC</t>
   </si>
   <si>
-    <t>006UW00000J8vsdYAB</t>
-  </si>
-  <si>
-    <t>006UW00000J957BYAR</t>
-  </si>
-  <si>
-    <t>006UW00000J8xxeYAB</t>
-  </si>
-  <si>
-    <t>006UW00000J8n2MYAR</t>
-  </si>
-  <si>
-    <t>006UW00000J8z3OYAR</t>
-  </si>
-  <si>
-    <t>006UW00000J8onuYAB</t>
-  </si>
-  <si>
-    <t>006UW00000Eq5I5YAJ</t>
-  </si>
-  <si>
-    <t>006f2000020MNkwAAG</t>
-  </si>
-  <si>
-    <t>006f200001wT0TAAA0</t>
-  </si>
-  <si>
-    <t>006f200001wUPDKAA4</t>
+    <t>006UW00000Izm6zYAB</t>
+  </si>
+  <si>
+    <t>ConnectWise, Inc.</t>
   </si>
   <si>
     <t>FourKites</t>
   </si>
   <si>
-    <t>ConnectWise, Inc.</t>
+    <t>STARLIMS</t>
   </si>
   <si>
     <t>Gibraltar Industries</t>
   </si>
   <si>
-    <t>STARLIMS</t>
-  </si>
-  <si>
     <t>Phoenix Lighting</t>
   </si>
   <si>
+    <t>Novata</t>
+  </si>
+  <si>
+    <t>Mansfield Sales Partners</t>
+  </si>
+  <si>
     <t>The Logic Factory</t>
   </si>
   <si>
-    <t>Hyland Software</t>
+    <t>Corcentric</t>
   </si>
   <si>
     <t>existing_client</t>
@@ -179,10 +170,10 @@
     <t>other</t>
   </si>
   <si>
+    <t>Enterprise</t>
+  </si>
+  <si>
     <t>Mid</t>
-  </si>
-  <si>
-    <t>Enterprise</t>
   </si>
   <si>
     <t>Commercial</t>
@@ -715,7 +706,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
@@ -731,7 +722,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>0.2250390348430733</v>
+        <v>0.2533451267444493</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -739,7 +730,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>0.1470393139152085</v>
+        <v>0.15617067187241</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -747,7 +738,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>0.1171130821825923</v>
+        <v>0.1319871285249258</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -755,7 +746,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>0.1024058130494268</v>
+        <v>0.1110763865295366</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -763,7 +754,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>0.07147905333501327</v>
+        <v>0.07276457990768948</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -771,7 +762,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>0.05552817469537897</v>
+        <v>0.06730149227878174</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -779,7 +770,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>0.04718950415150632</v>
+        <v>0.06130944119982024</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -787,7 +778,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>0.04307439337183125</v>
+        <v>0.03835124600237408</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -795,7 +786,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>0.0385347430558251</v>
+        <v>0.03173300116594579</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -803,7 +794,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>0.03481747703991296</v>
+        <v>0.0275776884781291</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -811,7 +802,7 @@
         <v>12</v>
       </c>
       <c r="B12">
-        <v>0.03017328864280967</v>
+        <v>0.02626054310731744</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -819,7 +810,7 @@
         <v>13</v>
       </c>
       <c r="B13">
-        <v>0.02678622779535138</v>
+        <v>0.01504375645521589</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -827,47 +818,7 @@
         <v>14</v>
       </c>
       <c r="B14">
-        <v>0.02073961448432277</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2">
-      <c r="A15" t="s">
-        <v>15</v>
-      </c>
-      <c r="B15">
-        <v>0.01988847508006411</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2">
-      <c r="A16" t="s">
-        <v>16</v>
-      </c>
-      <c r="B16">
-        <v>0.01342263327492355</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2">
-      <c r="A17" t="s">
-        <v>17</v>
-      </c>
-      <c r="B17">
-        <v>0.005118467697947223</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2">
-      <c r="A18" t="s">
-        <v>18</v>
-      </c>
-      <c r="B18">
-        <v>0.001598513472452824</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2">
-      <c r="A19" t="s">
-        <v>19</v>
-      </c>
-      <c r="B19">
-        <v>5.218991235979654E-05</v>
+        <v>0.00707893773340461</v>
       </c>
     </row>
   </sheetData>
@@ -882,10 +833,10 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B1" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="C1" t="s">
         <v>4</v>
@@ -897,407 +848,407 @@
         <v>5</v>
       </c>
       <c r="F1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>372.61</v>
       </c>
       <c r="D2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="E2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="F2">
-        <v>0.8393138291805022</v>
+        <v>0.836025813902403</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E3" t="s">
         <v>50</v>
       </c>
-      <c r="E3" t="s">
-        <v>52</v>
-      </c>
       <c r="F3">
-        <v>0.8393138291805022</v>
+        <v>0.8073787944033163</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C4">
         <v>0</v>
       </c>
       <c r="D4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E4" t="s">
         <v>50</v>
       </c>
-      <c r="E4" t="s">
-        <v>52</v>
-      </c>
       <c r="F4">
-        <v>0.8393138291805022</v>
+        <v>0.8073787944033163</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="C5">
-        <v>372.61</v>
+        <v>0</v>
       </c>
       <c r="D5" t="s">
+        <v>47</v>
+      </c>
+      <c r="E5" t="s">
         <v>50</v>
       </c>
-      <c r="E5" t="s">
-        <v>53</v>
-      </c>
       <c r="F5">
-        <v>0.8325045429045881</v>
+        <v>0.8073787944033163</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B6" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="C6">
-        <v>1839</v>
+        <v>28661</v>
       </c>
       <c r="D6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F6">
-        <v>0.8041537769094812</v>
+        <v>0.801113566299793</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="B7" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C7">
-        <v>0</v>
+        <v>1839</v>
       </c>
       <c r="D7" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E7" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="F7">
-        <v>0.8036096763211941</v>
+        <v>0.7763920325198355</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B8" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C8">
         <v>0</v>
       </c>
       <c r="D8" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E8" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F8">
-        <v>0.8036096763211941</v>
+        <v>0.7594348343070234</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B9" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="C9">
-        <v>28661</v>
+        <v>0</v>
       </c>
       <c r="D9" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E9" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="F9">
-        <v>0.7906190758627344</v>
+        <v>0.7594348343070234</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B10" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C10">
         <v>0</v>
       </c>
       <c r="D10" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="E10" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F10">
-        <v>0.7667258950033126</v>
+        <v>0.7421665549378333</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B11" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11">
+        <v>126</v>
+      </c>
+      <c r="D11" t="s">
         <v>48</v>
       </c>
-      <c r="C11">
-        <v>0</v>
-      </c>
-      <c r="D11" t="s">
-        <v>50</v>
-      </c>
       <c r="E11" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="F11">
-        <v>0.7413203617954394</v>
+        <v>0.7061727399865838</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B12" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C12">
-        <v>135</v>
+        <v>104</v>
       </c>
       <c r="D12" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E12" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="F12">
-        <v>0.7335526838015001</v>
+        <v>0.7061727399865838</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B13" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C13">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="D13" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E13" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="F13">
-        <v>0.7335526838015001</v>
+        <v>0.7057560733199171</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B14" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C14">
         <v>135</v>
       </c>
       <c r="D14" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E14" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="F14">
-        <v>0.7335526838015001</v>
+        <v>0.7057560733199171</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B15" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C15">
-        <v>104</v>
+        <v>181</v>
       </c>
       <c r="D15" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E15" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="F15">
-        <v>0.7335526838015001</v>
+        <v>0.7052591789099794</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B16" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C16">
         <v>217</v>
       </c>
       <c r="D16" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E16" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="F16">
-        <v>0.7320549879489655</v>
+        <v>0.7052591789099794</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C17">
-        <v>181</v>
+        <v>963</v>
       </c>
       <c r="D17" t="s">
+        <v>47</v>
+      </c>
+      <c r="E17" t="s">
         <v>51</v>
       </c>
-      <c r="E17" t="s">
-        <v>53</v>
-      </c>
       <c r="F17">
-        <v>0.7320549879489655</v>
+        <v>0.7037590164813601</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B18" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C18">
-        <v>5022.25</v>
+        <v>0</v>
       </c>
       <c r="D18" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="E18" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F18">
-        <v>0.7009191532278335</v>
+        <v>0.690555854449628</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B19" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C19">
         <v>0</v>
       </c>
       <c r="D19" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="E19" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F19">
-        <v>0.6916482120854046</v>
+        <v>0.690555854449628</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B20" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C20">
         <v>0</v>
       </c>
       <c r="D20" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="E20" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F20">
-        <v>0.6916482120854046</v>
+        <v>0.6898337791880755</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B21" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C21">
-        <v>0</v>
+        <v>1280</v>
       </c>
       <c r="D21" t="s">
+        <v>48</v>
+      </c>
+      <c r="E21" t="s">
         <v>50</v>
       </c>
-      <c r="E21" t="s">
-        <v>53</v>
-      </c>
       <c r="F21">
-        <v>0.6916482120854046</v>
+        <v>0.6886758463940779</v>
       </c>
     </row>
   </sheetData>
@@ -1312,24 +1263,24 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" t="s">
         <v>55</v>
       </c>
-      <c r="B1" t="s">
+      <c r="E1" t="s">
         <v>56</v>
-      </c>
-      <c r="C1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D1" t="s">
-        <v>58</v>
-      </c>
-      <c r="E1" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B2">
         <v>283</v>
@@ -1346,7 +1297,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B3">
         <v>526</v>
@@ -1363,7 +1314,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B4">
         <v>732</v>
@@ -1380,7 +1331,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B5">
         <v>3256</v>
@@ -1410,24 +1361,24 @@
         <v>3</v>
       </c>
       <c r="B1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E1" t="s">
         <v>64</v>
       </c>
-      <c r="C1" t="s">
+      <c r="F1" t="s">
         <v>65</v>
-      </c>
-      <c r="D1" t="s">
-        <v>66</v>
-      </c>
-      <c r="E1" t="s">
-        <v>67</v>
-      </c>
-      <c r="F1" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B2">
         <v>26</v>
@@ -1447,7 +1398,7 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B3">
         <v>69.78525641025641</v>
@@ -1467,7 +1418,7 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B4">
         <v>93.84722222222223</v>
@@ -1487,7 +1438,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B5">
         <v>86.06779661016949</v>
@@ -1507,7 +1458,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B6">
         <v>74.41666666666667</v>
@@ -1527,7 +1478,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B7">
         <v>72.8</v>
@@ -1547,7 +1498,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B8">
         <v>72</v>
@@ -1567,7 +1518,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B9">
         <v>130.8</v>
@@ -1587,7 +1538,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B10">
         <v>99.14285714285714</v>
@@ -1607,7 +1558,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B11">
         <v>262</v>
@@ -1637,18 +1588,18 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B1" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C1" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B2">
         <v>94</v>
@@ -1659,7 +1610,7 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B3">
         <v>18</v>
@@ -1670,7 +1621,7 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B4">
         <v>8</v>
@@ -1681,7 +1632,7 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B5">
         <v>7</v>
@@ -1702,25 +1653,25 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D1" t="s">
+        <v>76</v>
+      </c>
+      <c r="E1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F1" t="s">
         <v>83</v>
       </c>
-      <c r="B1" t="s">
-        <v>78</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="G1" t="s">
         <v>84</v>
-      </c>
-      <c r="D1" t="s">
-        <v>79</v>
-      </c>
-      <c r="E1" t="s">
-        <v>85</v>
-      </c>
-      <c r="F1" t="s">
-        <v>86</v>
-      </c>
-      <c r="G1" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -1784,33 +1735,33 @@
         <v>5</v>
       </c>
       <c r="B1" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C1" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D1" t="s">
+        <v>81</v>
+      </c>
+      <c r="E1" t="s">
+        <v>76</v>
+      </c>
+      <c r="F1" t="s">
+        <v>83</v>
+      </c>
+      <c r="G1" t="s">
         <v>84</v>
       </c>
-      <c r="E1" t="s">
-        <v>79</v>
-      </c>
-      <c r="F1" t="s">
-        <v>86</v>
-      </c>
-      <c r="G1" t="s">
-        <v>87</v>
-      </c>
       <c r="H1" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C2">
         <v>26</v>
@@ -1833,10 +1784,10 @@
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B3" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C3">
         <v>1196</v>
@@ -1859,10 +1810,10 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B4" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C4">
         <v>174</v>
@@ -1885,10 +1836,10 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B5" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C5">
         <v>242</v>
@@ -1911,10 +1862,10 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B6" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C6">
         <v>356</v>
@@ -1937,10 +1888,10 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B7" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C7">
         <v>184</v>
@@ -1963,10 +1914,10 @@
     </row>
     <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B8" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C8">
         <v>350</v>
@@ -1989,10 +1940,10 @@
     </row>
     <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B9" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C9">
         <v>388</v>
@@ -2015,10 +1966,10 @@
     </row>
     <row r="10" spans="1:8">
       <c r="A10" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B10" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C10">
         <v>9</v>
@@ -2051,36 +2002,36 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B1" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D1" t="s">
+        <v>76</v>
+      </c>
+      <c r="E1" t="s">
+        <v>82</v>
+      </c>
+      <c r="F1" t="s">
+        <v>83</v>
+      </c>
+      <c r="G1" t="s">
+        <v>90</v>
+      </c>
+      <c r="H1" t="s">
         <v>84</v>
       </c>
-      <c r="D1" t="s">
-        <v>79</v>
-      </c>
-      <c r="E1" t="s">
-        <v>85</v>
-      </c>
-      <c r="F1" t="s">
-        <v>86</v>
-      </c>
-      <c r="G1" t="s">
-        <v>93</v>
-      </c>
-      <c r="H1" t="s">
-        <v>87</v>
-      </c>
       <c r="I1" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B2">
         <v>75</v>
@@ -2109,7 +2060,7 @@
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B3">
         <v>27</v>
@@ -2138,7 +2089,7 @@
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B4">
         <v>38</v>
@@ -2167,7 +2118,7 @@
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B5">
         <v>62</v>
@@ -2196,7 +2147,7 @@
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B6">
         <v>56</v>
@@ -2225,7 +2176,7 @@
     </row>
     <row r="7" spans="1:9">
       <c r="A7" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B7">
         <v>56</v>
@@ -2254,7 +2205,7 @@
     </row>
     <row r="8" spans="1:9">
       <c r="A8" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B8">
         <v>55</v>
@@ -2283,7 +2234,7 @@
     </row>
     <row r="9" spans="1:9">
       <c r="A9" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B9">
         <v>57</v>
@@ -2312,7 +2263,7 @@
     </row>
     <row r="10" spans="1:9">
       <c r="A10" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B10">
         <v>84</v>
@@ -2341,7 +2292,7 @@
     </row>
     <row r="11" spans="1:9">
       <c r="A11" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B11">
         <v>86</v>
@@ -2370,7 +2321,7 @@
     </row>
     <row r="12" spans="1:9">
       <c r="A12" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B12">
         <v>108</v>
@@ -2399,7 +2350,7 @@
     </row>
     <row r="13" spans="1:9">
       <c r="A13" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B13">
         <v>92</v>
@@ -2428,7 +2379,7 @@
     </row>
     <row r="14" spans="1:9">
       <c r="A14" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B14">
         <v>68</v>
@@ -2457,7 +2408,7 @@
     </row>
     <row r="15" spans="1:9">
       <c r="A15" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B15">
         <v>90</v>
@@ -2486,7 +2437,7 @@
     </row>
     <row r="16" spans="1:9">
       <c r="A16" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B16">
         <v>86</v>
@@ -2515,7 +2466,7 @@
     </row>
     <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B17">
         <v>102</v>
@@ -2544,7 +2495,7 @@
     </row>
     <row r="18" spans="1:9">
       <c r="A18" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B18">
         <v>134</v>
@@ -2573,7 +2524,7 @@
     </row>
     <row r="19" spans="1:9">
       <c r="A19" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B19">
         <v>124</v>
@@ -2602,7 +2553,7 @@
     </row>
     <row r="20" spans="1:9">
       <c r="A20" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B20">
         <v>162</v>
@@ -2631,7 +2582,7 @@
     </row>
     <row r="21" spans="1:9">
       <c r="A21" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B21">
         <v>156</v>
@@ -2660,7 +2611,7 @@
     </row>
     <row r="22" spans="1:9">
       <c r="A22" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B22">
         <v>167</v>
@@ -2689,7 +2640,7 @@
     </row>
     <row r="23" spans="1:9">
       <c r="A23" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B23">
         <v>179</v>
@@ -2718,7 +2669,7 @@
     </row>
     <row r="24" spans="1:9">
       <c r="A24" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B24">
         <v>308</v>
@@ -2747,7 +2698,7 @@
     </row>
     <row r="25" spans="1:9">
       <c r="A25" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B25">
         <v>291</v>
@@ -2776,7 +2727,7 @@
     </row>
     <row r="26" spans="1:9">
       <c r="A26" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B26">
         <v>308</v>
@@ -2805,7 +2756,7 @@
     </row>
     <row r="27" spans="1:9">
       <c r="A27" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B27">
         <v>313</v>

</xml_diff>

<commit_message>
Rebuild dashboard with content-preserving React experience
</commit_message>
<xml_diff>
--- a/outputs/analysis/advanced_analytics.xlsx
+++ b/outputs/analysis/advanced_analytics.xlsx
@@ -1056,7 +1056,7 @@
         <v>71</v>
       </c>
       <c r="G2">
-        <v>0.7733831110668793</v>
+        <v>0.7733831110668794</v>
       </c>
       <c r="H2" t="s">
         <v>74</v>
@@ -1082,7 +1082,7 @@
         <v>71</v>
       </c>
       <c r="G3">
-        <v>0.7584242825937596</v>
+        <v>0.7584242825937598</v>
       </c>
       <c r="H3" t="s">
         <v>74</v>
@@ -1238,7 +1238,7 @@
         <v>71</v>
       </c>
       <c r="G9">
-        <v>0.7391946960238087</v>
+        <v>0.7391946960238088</v>
       </c>
       <c r="H9" t="s">
         <v>74</v>
@@ -1316,7 +1316,7 @@
         <v>72</v>
       </c>
       <c r="G12">
-        <v>0.7222770753936163</v>
+        <v>0.7222770753936161</v>
       </c>
       <c r="H12" t="s">
         <v>74</v>
@@ -1342,7 +1342,7 @@
         <v>73</v>
       </c>
       <c r="G13">
-        <v>0.7166722139896514</v>
+        <v>0.7166722139896516</v>
       </c>
       <c r="H13" t="s">
         <v>75</v>
@@ -1368,7 +1368,7 @@
         <v>71</v>
       </c>
       <c r="G14">
-        <v>0.708543887663886</v>
+        <v>0.7085438876638861</v>
       </c>
       <c r="H14" t="s">
         <v>75</v>

</xml_diff>

<commit_message>
Polish dashboard evidence interactions and accessibility
</commit_message>
<xml_diff>
--- a/outputs/analysis/advanced_analytics.xlsx
+++ b/outputs/analysis/advanced_analytics.xlsx
@@ -991,7 +991,7 @@
         <v>19</v>
       </c>
       <c r="Q2">
-        <v>0.06537146047494578</v>
+        <v>0.0653714604749458</v>
       </c>
       <c r="R2">
         <v>0.1394232562769266</v>
@@ -2398,7 +2398,7 @@
         <v>0.1578947368421053</v>
       </c>
       <c r="E2">
-        <v>0.000478322961440264</v>
+        <v>0.0004783229614402362</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -2432,7 +2432,7 @@
         <v>0.2123893805309734</v>
       </c>
       <c r="E4">
-        <v>0.1126510910919915</v>
+        <v>0.1126510910919916</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -2583,7 +2583,7 @@
         <v>83</v>
       </c>
       <c r="G2">
-        <v>0.7733831110668794</v>
+        <v>0.7733831110668795</v>
       </c>
       <c r="H2" t="s">
         <v>86</v>
@@ -2687,7 +2687,7 @@
         <v>84</v>
       </c>
       <c r="G6">
-        <v>0.7410267602055233</v>
+        <v>0.741026760205523</v>
       </c>
       <c r="H6" t="s">
         <v>86</v>
@@ -2713,7 +2713,7 @@
         <v>83</v>
       </c>
       <c r="G7">
-        <v>0.7408532634654529</v>
+        <v>0.740853263465453</v>
       </c>
       <c r="H7" t="s">
         <v>87</v>
@@ -2791,7 +2791,7 @@
         <v>84</v>
       </c>
       <c r="G10">
-        <v>0.7391186414334947</v>
+        <v>0.7391186414334949</v>
       </c>
       <c r="H10" t="s">
         <v>86</v>
@@ -2817,7 +2817,7 @@
         <v>84</v>
       </c>
       <c r="G11">
-        <v>0.7338072971228524</v>
+        <v>0.7338072971228526</v>
       </c>
       <c r="H11" t="s">
         <v>86</v>
@@ -2843,7 +2843,7 @@
         <v>84</v>
       </c>
       <c r="G12">
-        <v>0.7222770753936162</v>
+        <v>0.7222770753936161</v>
       </c>
       <c r="H12" t="s">
         <v>86</v>
@@ -2895,7 +2895,7 @@
         <v>83</v>
       </c>
       <c r="G14">
-        <v>0.7085438876638861</v>
+        <v>0.708543887663886</v>
       </c>
       <c r="H14" t="s">
         <v>87</v>
@@ -2973,7 +2973,7 @@
         <v>84</v>
       </c>
       <c r="G17">
-        <v>0.7016406634623603</v>
+        <v>0.7016406634623601</v>
       </c>
       <c r="H17" t="s">
         <v>87</v>
@@ -2999,7 +2999,7 @@
         <v>84</v>
       </c>
       <c r="G18">
-        <v>0.7016406634623603</v>
+        <v>0.7016406634623601</v>
       </c>
       <c r="H18" t="s">
         <v>87</v>
@@ -3025,7 +3025,7 @@
         <v>84</v>
       </c>
       <c r="G19">
-        <v>0.7016406634623603</v>
+        <v>0.7016406634623601</v>
       </c>
       <c r="H19" t="s">
         <v>87</v>
@@ -3051,7 +3051,7 @@
         <v>84</v>
       </c>
       <c r="G20">
-        <v>0.7016406634623603</v>
+        <v>0.7016406634623601</v>
       </c>
       <c r="H20" t="s">
         <v>87</v>
@@ -3077,7 +3077,7 @@
         <v>84</v>
       </c>
       <c r="G21">
-        <v>0.7016406634623603</v>
+        <v>0.7016406634623601</v>
       </c>
       <c r="H21" t="s">
         <v>87</v>

</xml_diff>

<commit_message>
Rebuild CMO evidence dashboard and browser deck
</commit_message>
<xml_diff>
--- a/outputs/analysis/advanced_analytics.xlsx
+++ b/outputs/analysis/advanced_analytics.xlsx
@@ -2635,7 +2635,7 @@
         <v>84</v>
       </c>
       <c r="G4">
-        <v>0.757367848721661</v>
+        <v>0.7573678487216609</v>
       </c>
       <c r="H4" t="s">
         <v>86</v>
@@ -2661,7 +2661,7 @@
         <v>84</v>
       </c>
       <c r="G5">
-        <v>0.7430330869295463</v>
+        <v>0.7430330869295462</v>
       </c>
       <c r="H5" t="s">
         <v>86</v>
@@ -2687,7 +2687,7 @@
         <v>84</v>
       </c>
       <c r="G6">
-        <v>0.741026760205523</v>
+        <v>0.7410267602055229</v>
       </c>
       <c r="H6" t="s">
         <v>86</v>
@@ -2765,7 +2765,7 @@
         <v>83</v>
       </c>
       <c r="G9">
-        <v>0.7391946960238088</v>
+        <v>0.7391946960238087</v>
       </c>
       <c r="H9" t="s">
         <v>86</v>
@@ -2791,7 +2791,7 @@
         <v>84</v>
       </c>
       <c r="G10">
-        <v>0.7391186414334949</v>
+        <v>0.7391186414334947</v>
       </c>
       <c r="H10" t="s">
         <v>86</v>
@@ -2895,7 +2895,7 @@
         <v>83</v>
       </c>
       <c r="G14">
-        <v>0.708543887663886</v>
+        <v>0.7085438876638861</v>
       </c>
       <c r="H14" t="s">
         <v>87</v>

</xml_diff>

<commit_message>
Integrate findings deck with legacy dashboard shell
</commit_message>
<xml_diff>
--- a/outputs/analysis/advanced_analytics.xlsx
+++ b/outputs/analysis/advanced_analytics.xlsx
@@ -991,7 +991,7 @@
         <v>19</v>
       </c>
       <c r="Q2">
-        <v>0.0653714604749458</v>
+        <v>0.06537146047494578</v>
       </c>
       <c r="R2">
         <v>0.1394232562769266</v>
@@ -2398,7 +2398,7 @@
         <v>0.1578947368421053</v>
       </c>
       <c r="E2">
-        <v>0.0004783229614402362</v>
+        <v>0.000478322961440264</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -2432,7 +2432,7 @@
         <v>0.2123893805309734</v>
       </c>
       <c r="E4">
-        <v>0.1126510910919916</v>
+        <v>0.1126510910919915</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -2687,7 +2687,7 @@
         <v>84</v>
       </c>
       <c r="G6">
-        <v>0.7410267602055229</v>
+        <v>0.7410267602055233</v>
       </c>
       <c r="H6" t="s">
         <v>86</v>
@@ -2713,7 +2713,7 @@
         <v>83</v>
       </c>
       <c r="G7">
-        <v>0.740853263465453</v>
+        <v>0.7408532634654529</v>
       </c>
       <c r="H7" t="s">
         <v>87</v>
@@ -2739,7 +2739,7 @@
         <v>84</v>
       </c>
       <c r="G8">
-        <v>0.7405346644903104</v>
+        <v>0.7405346644903105</v>
       </c>
       <c r="H8" t="s">
         <v>86</v>
@@ -2765,7 +2765,7 @@
         <v>83</v>
       </c>
       <c r="G9">
-        <v>0.7391946960238087</v>
+        <v>0.7391946960238088</v>
       </c>
       <c r="H9" t="s">
         <v>86</v>
@@ -2791,7 +2791,7 @@
         <v>84</v>
       </c>
       <c r="G10">
-        <v>0.7391186414334947</v>
+        <v>0.7391186414334949</v>
       </c>
       <c r="H10" t="s">
         <v>86</v>

</xml_diff>